<commit_message>
Enhance Excel model (scenarios/dashboard/charts) + split keyboard drills Win/Mac
- 완성본 8시트 고급화: Cover·시나리오 토글(Base/Bull/Bear)·비율 대시보드·
  투자요약(투자의견 자동)·차트·조건부서식·이름정의. formulas 엔진 재검증
  (대차=0, 오류0, 시나리오 전환 5,068→7,385→2,462원 확인)
- 실습본도 고급 구조 반영(IFERROR로 빈칸 시 에러 방지)
- 키보드 드릴 Windows/macOS 2종 분리(⌘T·⌘방향키 등 Mac 단축키 반영)
- index 다운로드 섹션(4카드 2×2)·미리보기(시나리오 토글 표)·R0 링크 갱신

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/financial-modeling/downloads/3-statement-model-complete.xlsx
+++ b/financial-modeling/downloads/3-statement-model-complete.xlsx
@@ -1,32 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="가정" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IS" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BS" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CF" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="가정" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="IS" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="BS" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CF" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Ratios" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="DCF" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Output" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="SCN">가정!$E$1</definedName>
+    <definedName name="WACC">가정!$C$15</definedName>
+    <definedName name="TermG">가정!$C$16</definedName>
+    <definedName name="TaxRate">가정!$C$7</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
-    <numFmt numFmtId="166" formatCode="0.000"/>
-    <numFmt numFmtId="167" formatCode="#,##0&quot;원&quot;"/>
+  <numFmts count="5">
+    <numFmt numFmtId="164" formatCode="#,##0&quot;원&quot;"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
+    <numFmt numFmtId="167" formatCode="0.0&quot;x&quot;"/>
+    <numFmt numFmtId="168" formatCode="0.000"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,7 +47,25 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="FF1E4F38"/>
-      <sz val="13"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="FF888888"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF0000FF"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -49,12 +76,45 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF1E4F38"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF2563EB"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="FF2563EB"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF008000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF008000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF1E4F38"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
@@ -64,26 +124,9 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <i val="1"/>
       <color rgb="FF000000"/>
       <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="FF008000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="FF008000"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -100,8 +143,8 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="FF0000FF"/>
-      <sz val="10"/>
+      <color rgb="FF1E4F38"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="5">
@@ -113,12 +156,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1E4F38"/>
+        <fgColor rgb="FFFFF3C4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FF1E4F38"/>
       </patternFill>
     </fill>
     <fill>
@@ -139,7 +182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -147,91 +190,164 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="14" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -302,6 +418,234 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>매출 &amp; 영업이익 (억원)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'IS'!$C$3:$H$3</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'IS'!$C$4:$H$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'IS'!$C$3:$H$3</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'IS'!$C$8:$H$8</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>영업이익률 (%)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'IS'!$C$3:$H$3</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'IS'!$C$15:$H$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2520000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2520000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -594,217 +938,557 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:D17"/>
+  <dimension ref="B2:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>가정 (Assumptions)</t>
-        </is>
-      </c>
-    </row>
     <row r="2">
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>단위: 억원 · 주식수 백만주 · 파란 셀만 바꾸면 모델 전체가 갱신됩니다</t>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>3-STATEMENT FINANCIAL MODEL</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>항목</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>값</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>비고</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>매출성장률 (추정연도)</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>YoY, 추정연도 공통 적용</t>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>가상 제조업 · Initiation Model (교육용)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>매출원가율 (COGS/매출)</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="D5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>판매관리비율 (SG&amp;A/매출)</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>시나리오 선택 →</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>1=Base · 2=Bull · 3=Bear</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>법인세율</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>목  차</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>핵심 결과 (활성 시나리오)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Capex / 매출</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="D8" s="2" t="inlineStr"/>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>① 가정 &amp; 시나리오</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>시나리오</t>
+        </is>
+      </c>
+      <c r="G8" s="9">
+        <f>Output!C4</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>감가상각률 (기초 유형자산 대비)</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D9" s="2" t="inlineStr"/>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>② 손익계산서 (IS)</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>목표주가</t>
+        </is>
+      </c>
+      <c r="G9" s="10">
+        <f>Output!C7</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>매출채권 회수기간 DSO (일)</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>③ 재무상태표 (BS)</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>현재주가</t>
+        </is>
+      </c>
+      <c r="G10" s="11">
+        <f>Output!C8</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>재고자산 보유기간 DIO (일)</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>60</v>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>④ 현금흐름표 (CF)</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>상승여력</t>
+        </is>
+      </c>
+      <c r="G11" s="12">
+        <f>Output!C9</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>매입채무 지급기간 DPO (일)</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="n">
-        <v>40</v>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>⑤ 재무비율 대시보드</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>투자의견</t>
+        </is>
+      </c>
+      <c r="G12" s="13">
+        <f>Output!C10</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>배당성향</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>⑥ DCF 밸류에이션</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>차입금 이자율</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>기초 차입금 기준</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>WACC (할인율)</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>영구성장률 g</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>&lt; WACC</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>주식수 (백만주)</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="n">
-        <v>50</v>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>⑦ 투자 요약</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId7"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002563EB"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:G17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>가정 &amp; 시나리오 (Assumptions)</t>
+        </is>
+      </c>
+      <c r="D1" s="15" t="inlineStr">
+        <is>
+          <t>시나리오</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>1=Base 2=Bull 3=Bear</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>파랑=입력 · 활성값(C열)=CHOOSE로 시나리오 전환 · 단위: 억원</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>항목</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>활성값</t>
+        </is>
+      </c>
+      <c r="D3" s="17" t="inlineStr">
+        <is>
+          <t>①Base</t>
+        </is>
+      </c>
+      <c r="E3" s="17" t="inlineStr">
+        <is>
+          <t>②Bull</t>
+        </is>
+      </c>
+      <c r="F3" s="17" t="inlineStr">
+        <is>
+          <t>③Bear</t>
+        </is>
+      </c>
+      <c r="G3" s="16" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>매출성장률 (추정)</t>
+        </is>
+      </c>
+      <c r="C4" s="18">
+        <f>CHOOSE($E$1,D4,E4,F4)</f>
+        <v/>
+      </c>
+      <c r="D4" s="19" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="E4" s="20" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F4" s="20" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>YoY</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>매출원가율</t>
+        </is>
+      </c>
+      <c r="C5" s="18">
+        <f>CHOOSE($E$1,D5,E5,F5)</f>
+        <v/>
+      </c>
+      <c r="D5" s="19" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="E5" s="20" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F5" s="20" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>판매관리비율</t>
+        </is>
+      </c>
+      <c r="C6" s="18">
+        <f>CHOOSE($E$1,D6,E6,F6)</f>
+        <v/>
+      </c>
+      <c r="D6" s="19" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E6" s="20" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F6" s="20" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="G6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>법인세율</t>
+        </is>
+      </c>
+      <c r="C7" s="18">
+        <f>CHOOSE($E$1,D7,E7,F7)</f>
+        <v/>
+      </c>
+      <c r="D7" s="19" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="E7" s="20" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F7" s="20" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="G7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Capex / 매출</t>
+        </is>
+      </c>
+      <c r="C8" s="18">
+        <f>CHOOSE($E$1,D8,E8,F8)</f>
+        <v/>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E8" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F8" s="20" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>감가상각률</t>
+        </is>
+      </c>
+      <c r="C9" s="18">
+        <f>CHOOSE($E$1,D9,E9,F9)</f>
+        <v/>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E9" s="20" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F9" s="20" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>기초 유형자산 대비</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>매출채권 DSO(일)</t>
+        </is>
+      </c>
+      <c r="C10" s="21">
+        <f>CHOOSE($E$1,D10,E10,F10)</f>
+        <v/>
+      </c>
+      <c r="D10" s="22" t="n">
+        <v>45</v>
+      </c>
+      <c r="E10" s="23" t="n">
+        <v>40</v>
+      </c>
+      <c r="F10" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="G10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>재고자산 DIO(일)</t>
+        </is>
+      </c>
+      <c r="C11" s="21">
+        <f>CHOOSE($E$1,D11,E11,F11)</f>
+        <v/>
+      </c>
+      <c r="D11" s="22" t="n">
+        <v>60</v>
+      </c>
+      <c r="E11" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="F11" s="23" t="n">
+        <v>70</v>
+      </c>
+      <c r="G11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>매입채무 DPO(일)</t>
+        </is>
+      </c>
+      <c r="C12" s="21">
+        <f>CHOOSE($E$1,D12,E12,F12)</f>
+        <v/>
+      </c>
+      <c r="D12" s="22" t="n">
+        <v>40</v>
+      </c>
+      <c r="E12" s="23" t="n">
+        <v>45</v>
+      </c>
+      <c r="F12" s="23" t="n">
+        <v>35</v>
+      </c>
+      <c r="G12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>배당성향</t>
+        </is>
+      </c>
+      <c r="C13" s="18">
+        <f>CHOOSE($E$1,D13,E13,F13)</f>
+        <v/>
+      </c>
+      <c r="D13" s="19" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E13" s="20" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F13" s="20" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G13" s="5" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>차입금 이자율</t>
+        </is>
+      </c>
+      <c r="C14" s="18">
+        <f>CHOOSE($E$1,D14,E14,F14)</f>
+        <v/>
+      </c>
+      <c r="D14" s="19" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="E14" s="20" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F14" s="20" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="G14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>WACC</t>
+        </is>
+      </c>
+      <c r="C15" s="18">
+        <f>CHOOSE($E$1,D15,E15,F15)</f>
+        <v/>
+      </c>
+      <c r="D15" s="19" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="E15" s="20" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="F15" s="20" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>영구성장률 g</t>
+        </is>
+      </c>
+      <c r="C16" s="18">
+        <f>CHOOSE($E$1,D16,E16,F16)</f>
+        <v/>
+      </c>
+      <c r="D16" s="19" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E16" s="20" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="F16" s="20" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>&lt; WACC</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>주식수(백만주)</t>
+        </is>
+      </c>
+      <c r="C17" s="24">
+        <f>CHOOSE($E$1,D17,E17,F17)</f>
+        <v/>
+      </c>
+      <c r="D17" s="25" t="n">
+        <v>50</v>
+      </c>
+      <c r="E17" s="26" t="n">
+        <v>50</v>
+      </c>
+      <c r="F17" s="26" t="n">
+        <v>50</v>
+      </c>
+      <c r="G17" s="5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="E1" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"1,2,3"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00217346"/>
@@ -814,7 +1498,7 @@
   <dimension ref="B1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
@@ -824,348 +1508,375 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>손익계산서 (Income Statement)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>단위: 억원</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>2022A</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>2023A</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>2024A</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="17" t="inlineStr">
         <is>
           <t>2025E</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="17" t="inlineStr">
         <is>
           <t>2026E</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="17" t="inlineStr">
         <is>
           <t>2027E</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>매출액</t>
         </is>
       </c>
-      <c r="C4" s="10" t="n">
+      <c r="C4" s="27" t="n">
         <v>1000</v>
       </c>
-      <c r="D4" s="10" t="n">
+      <c r="D4" s="27" t="n">
         <v>1120</v>
       </c>
-      <c r="E4" s="10" t="n">
+      <c r="E4" s="27" t="n">
         <v>1230</v>
       </c>
-      <c r="F4" s="11">
+      <c r="F4" s="28">
         <f>E4*(1+가정!$C$4)</f>
         <v/>
       </c>
-      <c r="G4" s="11">
+      <c r="G4" s="28">
         <f>F4*(1+가정!$C$4)</f>
         <v/>
       </c>
-      <c r="H4" s="11">
+      <c r="H4" s="28">
         <f>G4*(1+가정!$C$4)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>(-) 매출원가</t>
         </is>
       </c>
-      <c r="C5" s="10" t="n">
+      <c r="C5" s="27" t="n">
         <v>620</v>
       </c>
-      <c r="D5" s="10" t="n">
+      <c r="D5" s="27" t="n">
         <v>694</v>
       </c>
-      <c r="E5" s="10" t="n">
+      <c r="E5" s="27" t="n">
         <v>763</v>
       </c>
-      <c r="F5" s="12">
+      <c r="F5" s="29">
         <f>F4*가정!$C$5</f>
         <v/>
       </c>
-      <c r="G5" s="12">
+      <c r="G5" s="29">
         <f>G4*가정!$C$5</f>
         <v/>
       </c>
-      <c r="H5" s="12">
+      <c r="H5" s="29">
         <f>H4*가정!$C$5</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>매출총이익</t>
         </is>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="30">
         <f>C4-C5</f>
         <v/>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="30">
         <f>D4-D5</f>
         <v/>
       </c>
-      <c r="E6" s="13">
+      <c r="E6" s="30">
         <f>E4-E5</f>
         <v/>
       </c>
-      <c r="F6" s="13">
+      <c r="F6" s="30">
         <f>F4-F5</f>
         <v/>
       </c>
-      <c r="G6" s="13">
+      <c r="G6" s="30">
         <f>G4-G5</f>
         <v/>
       </c>
-      <c r="H6" s="13">
+      <c r="H6" s="30">
         <f>H4-H5</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>(-) 판매관리비</t>
         </is>
       </c>
-      <c r="C7" s="10" t="n">
+      <c r="C7" s="27" t="n">
         <v>200</v>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="27" t="n">
         <v>224</v>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="E7" s="27" t="n">
         <v>246</v>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="29">
         <f>F4*가정!$C$6</f>
         <v/>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="29">
         <f>G4*가정!$C$6</f>
         <v/>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="29">
         <f>H4*가정!$C$6</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>영업이익 (EBIT)</t>
         </is>
       </c>
-      <c r="C8" s="13">
+      <c r="C8" s="30">
         <f>C6-C7</f>
         <v/>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="30">
         <f>D6-D7</f>
         <v/>
       </c>
-      <c r="E8" s="13">
+      <c r="E8" s="30">
         <f>E6-E7</f>
         <v/>
       </c>
-      <c r="F8" s="13">
+      <c r="F8" s="30">
         <f>F6-F7</f>
         <v/>
       </c>
-      <c r="G8" s="13">
+      <c r="G8" s="30">
         <f>G6-G7</f>
         <v/>
       </c>
-      <c r="H8" s="13">
+      <c r="H8" s="30">
         <f>H6-H7</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>(-) 이자비용</t>
         </is>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="27" t="n">
         <v>18</v>
       </c>
-      <c r="D9" s="10" t="n">
+      <c r="D9" s="27" t="n">
         <v>19</v>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="E9" s="27" t="n">
         <v>20</v>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="29">
         <f>가정!$C$14*BS!E14</f>
         <v/>
       </c>
-      <c r="G9" s="12">
+      <c r="G9" s="29">
         <f>가정!$C$14*BS!F14</f>
         <v/>
       </c>
-      <c r="H9" s="12">
+      <c r="H9" s="29">
         <f>가정!$C$14*BS!G14</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>세전이익</t>
         </is>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="31">
         <f>C8-C9</f>
         <v/>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="31">
         <f>D8-D9</f>
         <v/>
       </c>
-      <c r="E10" s="14">
+      <c r="E10" s="31">
         <f>E8-E9</f>
         <v/>
       </c>
-      <c r="F10" s="14">
+      <c r="F10" s="31">
         <f>F8-F9</f>
         <v/>
       </c>
-      <c r="G10" s="14">
+      <c r="G10" s="31">
         <f>G8-G9</f>
         <v/>
       </c>
-      <c r="H10" s="14">
+      <c r="H10" s="31">
         <f>H8-H9</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>(-) 법인세</t>
         </is>
       </c>
-      <c r="C11" s="10" t="n">
+      <c r="C11" s="27" t="n">
         <v>36</v>
       </c>
-      <c r="D11" s="10" t="n">
+      <c r="D11" s="27" t="n">
         <v>40</v>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E11" s="27" t="n">
         <v>44</v>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="29">
         <f>F10*가정!$C$7</f>
         <v/>
       </c>
-      <c r="G11" s="12">
+      <c r="G11" s="29">
         <f>G10*가정!$C$7</f>
         <v/>
       </c>
-      <c r="H11" s="12">
+      <c r="H11" s="29">
         <f>H10*가정!$C$7</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>당기순이익</t>
         </is>
       </c>
-      <c r="C12" s="13">
+      <c r="C12" s="30">
         <f>C10-C11</f>
         <v/>
       </c>
-      <c r="D12" s="13">
+      <c r="D12" s="30">
         <f>D10-D11</f>
         <v/>
       </c>
-      <c r="E12" s="13">
+      <c r="E12" s="30">
         <f>E10-E11</f>
         <v/>
       </c>
-      <c r="F12" s="13">
+      <c r="F12" s="30">
         <f>F10-F11</f>
         <v/>
       </c>
-      <c r="G12" s="13">
+      <c r="G12" s="30">
         <f>G10-G11</f>
         <v/>
       </c>
-      <c r="H12" s="13">
+      <c r="H12" s="30">
         <f>H10-H11</f>
         <v/>
       </c>
     </row>
+    <row r="14">
+      <c r="B14" s="32" t="inlineStr">
+        <is>
+          <t>매출성장률</t>
+        </is>
+      </c>
+      <c r="D14" s="33">
+        <f>IFERROR(D4/C4-1,"-")</f>
+        <v/>
+      </c>
+      <c r="E14" s="33">
+        <f>IFERROR(E4/D4-1,"-")</f>
+        <v/>
+      </c>
+      <c r="F14" s="33">
+        <f>IFERROR(F4/E4-1,"-")</f>
+        <v/>
+      </c>
+      <c r="G14" s="33">
+        <f>IFERROR(G4/F4-1,"-")</f>
+        <v/>
+      </c>
+      <c r="H14" s="33">
+        <f>IFERROR(H4/G4-1,"-")</f>
+        <v/>
+      </c>
+    </row>
     <row r="15">
-      <c r="B15" s="15" t="inlineStr">
+      <c r="B15" s="32" t="inlineStr">
         <is>
           <t>영업이익률</t>
         </is>
       </c>
-      <c r="C15" s="16">
-        <f>C8/C4</f>
-        <v/>
-      </c>
-      <c r="D15" s="16">
-        <f>D8/D4</f>
-        <v/>
-      </c>
-      <c r="E15" s="16">
-        <f>E8/E4</f>
-        <v/>
-      </c>
-      <c r="F15" s="16">
-        <f>F8/F4</f>
-        <v/>
-      </c>
-      <c r="G15" s="16">
-        <f>G8/G4</f>
-        <v/>
-      </c>
-      <c r="H15" s="16">
-        <f>H8/H4</f>
+      <c r="C15" s="33">
+        <f>IFERROR(C8/C4,"-")</f>
+        <v/>
+      </c>
+      <c r="D15" s="33">
+        <f>IFERROR(D8/D4,"-")</f>
+        <v/>
+      </c>
+      <c r="E15" s="33">
+        <f>IFERROR(E8/E4,"-")</f>
+        <v/>
+      </c>
+      <c r="F15" s="33">
+        <f>IFERROR(F8/F4,"-")</f>
+        <v/>
+      </c>
+      <c r="G15" s="33">
+        <f>IFERROR(G8/G4,"-")</f>
+        <v/>
+      </c>
+      <c r="H15" s="33">
+        <f>IFERROR(H8/H4,"-")</f>
         <v/>
       </c>
     </row>
@@ -1174,7 +1885,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00217346"/>
@@ -1194,462 +1905,467 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>재무상태표 (Balance Sheet)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>단위: 억원</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>2022A</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>2023A</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>2024A</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="17" t="inlineStr">
         <is>
           <t>2025E</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="17" t="inlineStr">
         <is>
           <t>2026E</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="17" t="inlineStr">
         <is>
           <t>2027E</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="17" t="inlineStr">
+      <c r="B5" s="34" t="inlineStr">
         <is>
           <t>[ 자산 ]</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>현금및현금성자산</t>
         </is>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="27" t="n">
         <v>344</v>
       </c>
-      <c r="D6" s="10" t="n">
+      <c r="D6" s="27" t="n">
         <v>419</v>
       </c>
-      <c r="E6" s="10" t="n">
+      <c r="E6" s="27" t="n">
         <v>508</v>
       </c>
-      <c r="F6" s="12">
+      <c r="F6" s="29">
         <f>CF!F24</f>
         <v/>
       </c>
-      <c r="G6" s="12">
+      <c r="G6" s="29">
         <f>CF!G24</f>
         <v/>
       </c>
-      <c r="H6" s="12">
+      <c r="H6" s="29">
         <f>CF!H24</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>매출채권</t>
         </is>
       </c>
-      <c r="C7" s="10" t="n">
+      <c r="C7" s="27" t="n">
         <v>123</v>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="27" t="n">
         <v>138</v>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="E7" s="27" t="n">
         <v>152</v>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="29">
         <f>IS!F4*가정!$C$10/365</f>
         <v/>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="29">
         <f>IS!G4*가정!$C$10/365</f>
         <v/>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="29">
         <f>IS!H4*가정!$C$10/365</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>재고자산</t>
         </is>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="27" t="n">
         <v>102</v>
       </c>
-      <c r="D8" s="10" t="n">
+      <c r="D8" s="27" t="n">
         <v>114</v>
       </c>
-      <c r="E8" s="10" t="n">
+      <c r="E8" s="27" t="n">
         <v>125</v>
       </c>
-      <c r="F8" s="12">
+      <c r="F8" s="29">
         <f>IS!F5*가정!$C$11/365</f>
         <v/>
       </c>
-      <c r="G8" s="12">
+      <c r="G8" s="29">
         <f>IS!G5*가정!$C$11/365</f>
         <v/>
       </c>
-      <c r="H8" s="12">
+      <c r="H8" s="29">
         <f>IS!H5*가정!$C$11/365</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>유형자산(순)</t>
         </is>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="27" t="n">
         <v>500</v>
       </c>
-      <c r="D9" s="10" t="n">
+      <c r="D9" s="27" t="n">
         <v>540</v>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="E9" s="27" t="n">
         <v>580</v>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="29">
         <f>E9+가정!$C$8*IS!F4-가정!$C$9*E9</f>
         <v/>
       </c>
-      <c r="G9" s="12">
+      <c r="G9" s="29">
         <f>F9+가정!$C$8*IS!G4-가정!$C$9*F9</f>
         <v/>
       </c>
-      <c r="H9" s="12">
+      <c r="H9" s="29">
         <f>G9+가정!$C$8*IS!H4-가정!$C$9*G9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>자산총계</t>
         </is>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="30">
         <f>SUM(C6:C9)</f>
         <v/>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="30">
         <f>SUM(D6:D9)</f>
         <v/>
       </c>
-      <c r="E10" s="13">
+      <c r="E10" s="30">
         <f>SUM(E6:E9)</f>
         <v/>
       </c>
-      <c r="F10" s="13">
+      <c r="F10" s="30">
         <f>SUM(F6:F9)</f>
         <v/>
       </c>
-      <c r="G10" s="13">
+      <c r="G10" s="30">
         <f>SUM(G6:G9)</f>
         <v/>
       </c>
-      <c r="H10" s="13">
+      <c r="H10" s="30">
         <f>SUM(H6:H9)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B12" s="34" t="inlineStr">
         <is>
           <t>[ 부채 ]</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>매입채무</t>
         </is>
       </c>
-      <c r="C13" s="10" t="n">
+      <c r="C13" s="27" t="n">
         <v>68</v>
       </c>
-      <c r="D13" s="10" t="n">
+      <c r="D13" s="27" t="n">
         <v>76</v>
       </c>
-      <c r="E13" s="10" t="n">
+      <c r="E13" s="27" t="n">
         <v>84</v>
       </c>
-      <c r="F13" s="12">
+      <c r="F13" s="29">
         <f>IS!F5*가정!$C$12/365</f>
         <v/>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="29">
         <f>IS!G5*가정!$C$12/365</f>
         <v/>
       </c>
-      <c r="H13" s="12">
+      <c r="H13" s="29">
         <f>IS!H5*가정!$C$12/365</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>차입금</t>
         </is>
       </c>
-      <c r="C14" s="10" t="n">
+      <c r="C14" s="27" t="n">
         <v>400</v>
       </c>
-      <c r="D14" s="10" t="n">
+      <c r="D14" s="27" t="n">
         <v>420</v>
       </c>
-      <c r="E14" s="10" t="n">
+      <c r="E14" s="27" t="n">
         <v>440</v>
       </c>
-      <c r="F14" s="14">
+      <c r="F14" s="31">
         <f>E14</f>
         <v/>
       </c>
-      <c r="G14" s="14">
+      <c r="G14" s="31">
         <f>F14</f>
         <v/>
       </c>
-      <c r="H14" s="14">
+      <c r="H14" s="31">
         <f>G14</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>부채총계</t>
         </is>
       </c>
-      <c r="C15" s="13">
+      <c r="C15" s="30">
         <f>SUM(C13:C14)</f>
         <v/>
       </c>
-      <c r="D15" s="13">
+      <c r="D15" s="30">
         <f>SUM(D13:D14)</f>
         <v/>
       </c>
-      <c r="E15" s="13">
+      <c r="E15" s="30">
         <f>SUM(E13:E14)</f>
         <v/>
       </c>
-      <c r="F15" s="13">
+      <c r="F15" s="30">
         <f>SUM(F13:F14)</f>
         <v/>
       </c>
-      <c r="G15" s="13">
+      <c r="G15" s="30">
         <f>SUM(G13:G14)</f>
         <v/>
       </c>
-      <c r="H15" s="13">
+      <c r="H15" s="30">
         <f>SUM(H13:H14)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="17" t="inlineStr">
+      <c r="B17" s="34" t="inlineStr">
         <is>
           <t>[ 자본 ]</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>자본금</t>
         </is>
       </c>
-      <c r="C18" s="10" t="n">
+      <c r="C18" s="27" t="n">
         <v>300</v>
       </c>
-      <c r="D18" s="10" t="n">
+      <c r="D18" s="27" t="n">
         <v>300</v>
       </c>
-      <c r="E18" s="10" t="n">
+      <c r="E18" s="27" t="n">
         <v>300</v>
       </c>
-      <c r="F18" s="14">
+      <c r="F18" s="31">
         <f>E18</f>
         <v/>
       </c>
-      <c r="G18" s="14">
+      <c r="G18" s="31">
         <f>F18</f>
         <v/>
       </c>
-      <c r="H18" s="14">
+      <c r="H18" s="31">
         <f>G18</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>이익잉여금</t>
         </is>
       </c>
-      <c r="C19" s="10" t="n">
+      <c r="C19" s="27" t="n">
         <v>301</v>
       </c>
-      <c r="D19" s="10" t="n">
+      <c r="D19" s="27" t="n">
         <v>415</v>
       </c>
-      <c r="E19" s="10" t="n">
+      <c r="E19" s="27" t="n">
         <v>541</v>
       </c>
-      <c r="F19" s="12">
+      <c r="F19" s="29">
         <f>E19+IS!F12-가정!$C$13*IS!F12</f>
         <v/>
       </c>
-      <c r="G19" s="12">
+      <c r="G19" s="29">
         <f>F19+IS!G12-가정!$C$13*IS!G12</f>
         <v/>
       </c>
-      <c r="H19" s="12">
+      <c r="H19" s="29">
         <f>G19+IS!H12-가정!$C$13*IS!H12</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>자본총계</t>
         </is>
       </c>
-      <c r="C20" s="13">
+      <c r="C20" s="30">
         <f>SUM(C18:C19)</f>
         <v/>
       </c>
-      <c r="D20" s="13">
+      <c r="D20" s="30">
         <f>SUM(D18:D19)</f>
         <v/>
       </c>
-      <c r="E20" s="13">
+      <c r="E20" s="30">
         <f>SUM(E18:E19)</f>
         <v/>
       </c>
-      <c r="F20" s="13">
+      <c r="F20" s="30">
         <f>SUM(F18:F19)</f>
         <v/>
       </c>
-      <c r="G20" s="13">
+      <c r="G20" s="30">
         <f>SUM(G18:G19)</f>
         <v/>
       </c>
-      <c r="H20" s="13">
+      <c r="H20" s="30">
         <f>SUM(H18:H19)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>부채와자본총계</t>
         </is>
       </c>
-      <c r="C21" s="13">
+      <c r="C21" s="30">
         <f>C15+C20</f>
         <v/>
       </c>
-      <c r="D21" s="13">
+      <c r="D21" s="30">
         <f>D15+D20</f>
         <v/>
       </c>
-      <c r="E21" s="13">
+      <c r="E21" s="30">
         <f>E15+E20</f>
         <v/>
       </c>
-      <c r="F21" s="13">
+      <c r="F21" s="30">
         <f>F15+F20</f>
         <v/>
       </c>
-      <c r="G21" s="13">
+      <c r="G21" s="30">
         <f>G15+G20</f>
         <v/>
       </c>
-      <c r="H21" s="13">
+      <c r="H21" s="30">
         <f>H15+H20</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B23" s="32" t="inlineStr">
         <is>
           <t>검증 (자산-부채-자본)</t>
         </is>
       </c>
-      <c r="C23" s="18">
+      <c r="C23" s="35">
         <f>C10-C21</f>
         <v/>
       </c>
-      <c r="D23" s="18">
+      <c r="D23" s="35">
         <f>D10-D21</f>
         <v/>
       </c>
-      <c r="E23" s="18">
+      <c r="E23" s="35">
         <f>E10-E21</f>
         <v/>
       </c>
-      <c r="F23" s="18">
+      <c r="F23" s="35">
         <f>F10-F21</f>
         <v/>
       </c>
-      <c r="G23" s="18">
+      <c r="G23" s="35">
         <f>G10-G21</f>
         <v/>
       </c>
-      <c r="H23" s="18">
+      <c r="H23" s="35">
         <f>H10-H21</f>
         <v/>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="C23:H23">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>ABS(C23)&gt;0.5</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00217346"/>
@@ -1669,339 +2385,339 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>현금흐름표 (Cash Flow, 간접법)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>단위: 억원 · 추정연도만 산출</t>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>단위: 억원 · 추정연도 산출</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>2022A</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>2023A</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>2024A</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="17" t="inlineStr">
         <is>
           <t>2025E</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="17" t="inlineStr">
         <is>
           <t>2026E</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="17" t="inlineStr">
         <is>
           <t>2027E</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="17" t="inlineStr">
+      <c r="B5" s="34" t="inlineStr">
         <is>
           <t>[ 영업활동 ]</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>당기순이익</t>
         </is>
       </c>
-      <c r="F6" s="12">
+      <c r="F6" s="29">
         <f>IS!F12</f>
         <v/>
       </c>
-      <c r="G6" s="12">
+      <c r="G6" s="29">
         <f>IS!G12</f>
         <v/>
       </c>
-      <c r="H6" s="12">
+      <c r="H6" s="29">
         <f>IS!H12</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>(+) 감가상각비</t>
         </is>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="29">
         <f>가정!$C$9*BS!E9</f>
         <v/>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="29">
         <f>가정!$C$9*BS!F9</f>
         <v/>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="29">
         <f>가정!$C$9*BS!G9</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>(-) 매출채권 증감</t>
         </is>
       </c>
-      <c r="F8" s="12">
+      <c r="F8" s="29">
         <f>-(BS!F7-BS!E7)</f>
         <v/>
       </c>
-      <c r="G8" s="12">
+      <c r="G8" s="29">
         <f>-(BS!G7-BS!F7)</f>
         <v/>
       </c>
-      <c r="H8" s="12">
+      <c r="H8" s="29">
         <f>-(BS!H7-BS!G7)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>(-) 재고자산 증감</t>
         </is>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="29">
         <f>-(BS!F8-BS!E8)</f>
         <v/>
       </c>
-      <c r="G9" s="12">
+      <c r="G9" s="29">
         <f>-(BS!G8-BS!F8)</f>
         <v/>
       </c>
-      <c r="H9" s="12">
+      <c r="H9" s="29">
         <f>-(BS!H8-BS!G8)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>(+) 매입채무 증감</t>
         </is>
       </c>
-      <c r="F10" s="12">
+      <c r="F10" s="29">
         <f>BS!F13-BS!E13</f>
         <v/>
       </c>
-      <c r="G10" s="12">
+      <c r="G10" s="29">
         <f>BS!G13-BS!F13</f>
         <v/>
       </c>
-      <c r="H10" s="12">
+      <c r="H10" s="29">
         <f>BS!H13-BS!G13</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>영업활동 현금흐름</t>
         </is>
       </c>
-      <c r="F11" s="13">
+      <c r="F11" s="30">
         <f>SUM(F6:F10)</f>
         <v/>
       </c>
-      <c r="G11" s="13">
+      <c r="G11" s="30">
         <f>SUM(G6:G10)</f>
         <v/>
       </c>
-      <c r="H11" s="13">
+      <c r="H11" s="30">
         <f>SUM(H6:H10)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="17" t="inlineStr">
+      <c r="B13" s="34" t="inlineStr">
         <is>
           <t>[ 투자활동 ]</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>(-) Capex</t>
         </is>
       </c>
-      <c r="F14" s="12">
+      <c r="F14" s="29">
         <f>-가정!$C$8*IS!F4</f>
         <v/>
       </c>
-      <c r="G14" s="12">
+      <c r="G14" s="29">
         <f>-가정!$C$8*IS!G4</f>
         <v/>
       </c>
-      <c r="H14" s="12">
+      <c r="H14" s="29">
         <f>-가정!$C$8*IS!H4</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>투자활동 현금흐름</t>
         </is>
       </c>
-      <c r="F15" s="13">
+      <c r="F15" s="30">
         <f>F14</f>
         <v/>
       </c>
-      <c r="G15" s="13">
+      <c r="G15" s="30">
         <f>G14</f>
         <v/>
       </c>
-      <c r="H15" s="13">
+      <c r="H15" s="30">
         <f>H14</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="17" t="inlineStr">
+      <c r="B17" s="34" t="inlineStr">
         <is>
           <t>[ 재무활동 ]</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>차입금 증감</t>
         </is>
       </c>
-      <c r="F18" s="12">
+      <c r="F18" s="29">
         <f>BS!F14-BS!E14</f>
         <v/>
       </c>
-      <c r="G18" s="12">
+      <c r="G18" s="29">
         <f>BS!G14-BS!F14</f>
         <v/>
       </c>
-      <c r="H18" s="12">
+      <c r="H18" s="29">
         <f>BS!H14-BS!G14</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>(-) 배당금</t>
         </is>
       </c>
-      <c r="F19" s="12">
+      <c r="F19" s="29">
         <f>-가정!$C$13*IS!F12</f>
         <v/>
       </c>
-      <c r="G19" s="12">
+      <c r="G19" s="29">
         <f>-가정!$C$13*IS!G12</f>
         <v/>
       </c>
-      <c r="H19" s="12">
+      <c r="H19" s="29">
         <f>-가정!$C$13*IS!H12</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>재무활동 현금흐름</t>
         </is>
       </c>
-      <c r="F20" s="13">
+      <c r="F20" s="30">
         <f>SUM(F18:F19)</f>
         <v/>
       </c>
-      <c r="G20" s="13">
+      <c r="G20" s="30">
         <f>SUM(G18:G19)</f>
         <v/>
       </c>
-      <c r="H20" s="13">
+      <c r="H20" s="30">
         <f>SUM(H18:H19)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>순현금흐름</t>
         </is>
       </c>
-      <c r="F22" s="13">
+      <c r="F22" s="30">
         <f>F11+F15+F20</f>
         <v/>
       </c>
-      <c r="G22" s="13">
+      <c r="G22" s="30">
         <f>G11+G15+G20</f>
         <v/>
       </c>
-      <c r="H22" s="13">
+      <c r="H22" s="30">
         <f>H11+H15+H20</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>기초 현금</t>
         </is>
       </c>
-      <c r="F23" s="12">
+      <c r="F23" s="29">
         <f>BS!E6</f>
         <v/>
       </c>
-      <c r="G23" s="12">
+      <c r="G23" s="29">
         <f>BS!F6</f>
         <v/>
       </c>
-      <c r="H23" s="12">
+      <c r="H23" s="29">
         <f>BS!G6</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>기말 현금</t>
         </is>
       </c>
-      <c r="F24" s="13">
+      <c r="F24" s="30">
         <f>F22+F23</f>
         <v/>
       </c>
-      <c r="G24" s="13">
+      <c r="G24" s="30">
         <f>G22+G23</f>
         <v/>
       </c>
-      <c r="H24" s="13">
+      <c r="H24" s="30">
         <f>H22+H23</f>
         <v/>
       </c>
@@ -2011,7 +2727,487 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="007C3AED"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:H18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>재무비율 대시보드</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>IS·BS에서 자동 산출</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>항목</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>2022A</t>
+        </is>
+      </c>
+      <c r="D3" s="17" t="inlineStr">
+        <is>
+          <t>2023A</t>
+        </is>
+      </c>
+      <c r="E3" s="17" t="inlineStr">
+        <is>
+          <t>2024A</t>
+        </is>
+      </c>
+      <c r="F3" s="17" t="inlineStr">
+        <is>
+          <t>2025E</t>
+        </is>
+      </c>
+      <c r="G3" s="17" t="inlineStr">
+        <is>
+          <t>2026E</t>
+        </is>
+      </c>
+      <c r="H3" s="17" t="inlineStr">
+        <is>
+          <t>2027E</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="34" t="inlineStr">
+        <is>
+          <t>[ 수익성 ]</t>
+        </is>
+      </c>
+      <c r="C4" s="36" t="inlineStr"/>
+      <c r="D4" s="36" t="inlineStr"/>
+      <c r="E4" s="36" t="inlineStr"/>
+      <c r="F4" s="36" t="inlineStr"/>
+      <c r="G4" s="36" t="inlineStr"/>
+      <c r="H4" s="36" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>매출총이익률</t>
+        </is>
+      </c>
+      <c r="C5" s="37">
+        <f>IFERROR(IS!C6/IS!C4,"-")</f>
+        <v/>
+      </c>
+      <c r="D5" s="37">
+        <f>IFERROR(IS!D6/IS!D4,"-")</f>
+        <v/>
+      </c>
+      <c r="E5" s="37">
+        <f>IFERROR(IS!E6/IS!E4,"-")</f>
+        <v/>
+      </c>
+      <c r="F5" s="37">
+        <f>IFERROR(IS!F6/IS!F4,"-")</f>
+        <v/>
+      </c>
+      <c r="G5" s="37">
+        <f>IFERROR(IS!G6/IS!G4,"-")</f>
+        <v/>
+      </c>
+      <c r="H5" s="37">
+        <f>IFERROR(IS!H6/IS!H4,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>영업이익률</t>
+        </is>
+      </c>
+      <c r="C6" s="37">
+        <f>IFERROR(IS!C8/IS!C4,"-")</f>
+        <v/>
+      </c>
+      <c r="D6" s="37">
+        <f>IFERROR(IS!D8/IS!D4,"-")</f>
+        <v/>
+      </c>
+      <c r="E6" s="37">
+        <f>IFERROR(IS!E8/IS!E4,"-")</f>
+        <v/>
+      </c>
+      <c r="F6" s="37">
+        <f>IFERROR(IS!F8/IS!F4,"-")</f>
+        <v/>
+      </c>
+      <c r="G6" s="37">
+        <f>IFERROR(IS!G8/IS!G4,"-")</f>
+        <v/>
+      </c>
+      <c r="H6" s="37">
+        <f>IFERROR(IS!H8/IS!H4,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>순이익률</t>
+        </is>
+      </c>
+      <c r="C7" s="37">
+        <f>IFERROR(IS!C12/IS!C4,"-")</f>
+        <v/>
+      </c>
+      <c r="D7" s="37">
+        <f>IFERROR(IS!D12/IS!D4,"-")</f>
+        <v/>
+      </c>
+      <c r="E7" s="37">
+        <f>IFERROR(IS!E12/IS!E4,"-")</f>
+        <v/>
+      </c>
+      <c r="F7" s="37">
+        <f>IFERROR(IS!F12/IS!F4,"-")</f>
+        <v/>
+      </c>
+      <c r="G7" s="37">
+        <f>IFERROR(IS!G12/IS!G4,"-")</f>
+        <v/>
+      </c>
+      <c r="H7" s="37">
+        <f>IFERROR(IS!H12/IS!H4,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>ROE</t>
+        </is>
+      </c>
+      <c r="C8" s="37">
+        <f>IFERROR(IS!C12/BS!C20,"-")</f>
+        <v/>
+      </c>
+      <c r="D8" s="37">
+        <f>IFERROR(IS!D12/BS!D20,"-")</f>
+        <v/>
+      </c>
+      <c r="E8" s="37">
+        <f>IFERROR(IS!E12/BS!E20,"-")</f>
+        <v/>
+      </c>
+      <c r="F8" s="37">
+        <f>IFERROR(IS!F12/BS!F20,"-")</f>
+        <v/>
+      </c>
+      <c r="G8" s="37">
+        <f>IFERROR(IS!G12/BS!G20,"-")</f>
+        <v/>
+      </c>
+      <c r="H8" s="37">
+        <f>IFERROR(IS!H12/BS!H20,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>ROA</t>
+        </is>
+      </c>
+      <c r="C9" s="37">
+        <f>IFERROR(IS!C12/BS!C10,"-")</f>
+        <v/>
+      </c>
+      <c r="D9" s="37">
+        <f>IFERROR(IS!D12/BS!D10,"-")</f>
+        <v/>
+      </c>
+      <c r="E9" s="37">
+        <f>IFERROR(IS!E12/BS!E10,"-")</f>
+        <v/>
+      </c>
+      <c r="F9" s="37">
+        <f>IFERROR(IS!F12/BS!F10,"-")</f>
+        <v/>
+      </c>
+      <c r="G9" s="37">
+        <f>IFERROR(IS!G12/BS!G10,"-")</f>
+        <v/>
+      </c>
+      <c r="H9" s="37">
+        <f>IFERROR(IS!H12/BS!H10,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="34" t="inlineStr">
+        <is>
+          <t>[ 성장성 ]</t>
+        </is>
+      </c>
+      <c r="C10" s="36" t="inlineStr"/>
+      <c r="D10" s="36" t="inlineStr"/>
+      <c r="E10" s="36" t="inlineStr"/>
+      <c r="F10" s="36" t="inlineStr"/>
+      <c r="G10" s="36" t="inlineStr"/>
+      <c r="H10" s="36" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>매출 YoY</t>
+        </is>
+      </c>
+      <c r="C11" s="37">
+        <f>IS!C14</f>
+        <v/>
+      </c>
+      <c r="D11" s="37">
+        <f>IS!D14</f>
+        <v/>
+      </c>
+      <c r="E11" s="37">
+        <f>IS!E14</f>
+        <v/>
+      </c>
+      <c r="F11" s="37">
+        <f>IS!F14</f>
+        <v/>
+      </c>
+      <c r="G11" s="37">
+        <f>IS!G14</f>
+        <v/>
+      </c>
+      <c r="H11" s="37">
+        <f>IS!H14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>영업이익 YoY</t>
+        </is>
+      </c>
+      <c r="C12" s="37">
+        <f>IFERROR(IS!C8/IS!C8-1,"-")</f>
+        <v/>
+      </c>
+      <c r="D12" s="37">
+        <f>IFERROR(IS!D8/IS!C8-1,"-")</f>
+        <v/>
+      </c>
+      <c r="E12" s="37">
+        <f>IFERROR(IS!E8/IS!D8-1,"-")</f>
+        <v/>
+      </c>
+      <c r="F12" s="37">
+        <f>IFERROR(IS!F8/IS!E8-1,"-")</f>
+        <v/>
+      </c>
+      <c r="G12" s="37">
+        <f>IFERROR(IS!G8/IS!F8-1,"-")</f>
+        <v/>
+      </c>
+      <c r="H12" s="37">
+        <f>IFERROR(IS!H8/IS!G8-1,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="34" t="inlineStr">
+        <is>
+          <t>[ 안정성 ]</t>
+        </is>
+      </c>
+      <c r="C13" s="36" t="inlineStr"/>
+      <c r="D13" s="36" t="inlineStr"/>
+      <c r="E13" s="36" t="inlineStr"/>
+      <c r="F13" s="36" t="inlineStr"/>
+      <c r="G13" s="36" t="inlineStr"/>
+      <c r="H13" s="36" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>부채비율</t>
+        </is>
+      </c>
+      <c r="C14" s="37">
+        <f>IFERROR(BS!C15/BS!C20,"-")</f>
+        <v/>
+      </c>
+      <c r="D14" s="37">
+        <f>IFERROR(BS!D15/BS!D20,"-")</f>
+        <v/>
+      </c>
+      <c r="E14" s="37">
+        <f>IFERROR(BS!E15/BS!E20,"-")</f>
+        <v/>
+      </c>
+      <c r="F14" s="37">
+        <f>IFERROR(BS!F15/BS!F20,"-")</f>
+        <v/>
+      </c>
+      <c r="G14" s="37">
+        <f>IFERROR(BS!G15/BS!G20,"-")</f>
+        <v/>
+      </c>
+      <c r="H14" s="37">
+        <f>IFERROR(BS!H15/BS!H20,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>이자보상배율</t>
+        </is>
+      </c>
+      <c r="C15" s="38">
+        <f>IFERROR(IS!C8/IS!C9,"-")</f>
+        <v/>
+      </c>
+      <c r="D15" s="38">
+        <f>IFERROR(IS!D8/IS!D9,"-")</f>
+        <v/>
+      </c>
+      <c r="E15" s="38">
+        <f>IFERROR(IS!E8/IS!E9,"-")</f>
+        <v/>
+      </c>
+      <c r="F15" s="38">
+        <f>IFERROR(IS!F8/IS!F9,"-")</f>
+        <v/>
+      </c>
+      <c r="G15" s="38">
+        <f>IFERROR(IS!G8/IS!G9,"-")</f>
+        <v/>
+      </c>
+      <c r="H15" s="38">
+        <f>IFERROR(IS!H8/IS!H9,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="34" t="inlineStr">
+        <is>
+          <t>[ 활동성 ]</t>
+        </is>
+      </c>
+      <c r="C16" s="36" t="inlineStr"/>
+      <c r="D16" s="36" t="inlineStr"/>
+      <c r="E16" s="36" t="inlineStr"/>
+      <c r="F16" s="36" t="inlineStr"/>
+      <c r="G16" s="36" t="inlineStr"/>
+      <c r="H16" s="36" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>매출채권 회전일</t>
+        </is>
+      </c>
+      <c r="C17" s="39">
+        <f>IFERROR(BS!C7/IS!C4*365,"-")</f>
+        <v/>
+      </c>
+      <c r="D17" s="39">
+        <f>IFERROR(BS!D7/IS!D4*365,"-")</f>
+        <v/>
+      </c>
+      <c r="E17" s="39">
+        <f>IFERROR(BS!E7/IS!E4*365,"-")</f>
+        <v/>
+      </c>
+      <c r="F17" s="39">
+        <f>IFERROR(BS!F7/IS!F4*365,"-")</f>
+        <v/>
+      </c>
+      <c r="G17" s="39">
+        <f>IFERROR(BS!G7/IS!G4*365,"-")</f>
+        <v/>
+      </c>
+      <c r="H17" s="39">
+        <f>IFERROR(BS!H7/IS!H4*365,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>재고 회전일</t>
+        </is>
+      </c>
+      <c r="C18" s="39">
+        <f>IFERROR(BS!C8/IS!C5*365,"-")</f>
+        <v/>
+      </c>
+      <c r="D18" s="39">
+        <f>IFERROR(BS!D8/IS!D5*365,"-")</f>
+        <v/>
+      </c>
+      <c r="E18" s="39">
+        <f>IFERROR(BS!E8/IS!E5*365,"-")</f>
+        <v/>
+      </c>
+      <c r="F18" s="39">
+        <f>IFERROR(BS!F8/IS!F5*365,"-")</f>
+        <v/>
+      </c>
+      <c r="G18" s="39">
+        <f>IFERROR(BS!G8/IS!G5*365,"-")</f>
+        <v/>
+      </c>
+      <c r="H18" s="39">
+        <f>IFERROR(BS!H8/IS!H5*365,"-")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="C5:H7">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="0010B981"/>
@@ -2021,7 +3217,7 @@
   <dimension ref="B1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -2031,473 +3227,603 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>DCF 밸류에이션</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>단위: 억원 · 주당가치 원</t>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>단위: 억원 · 주당 원</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>2025E</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>2026E</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>2027E</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>영업이익 (EBIT)</t>
         </is>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="29">
         <f>IS!F8</f>
         <v/>
       </c>
-      <c r="D4" s="12">
+      <c r="D4" s="29">
         <f>IS!G8</f>
         <v/>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="29">
         <f>IS!H8</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>EBIT×(1-t)</t>
         </is>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="29">
         <f>C4*(1-가정!$C$7)</f>
         <v/>
       </c>
-      <c r="D5" s="12">
+      <c r="D5" s="29">
         <f>D4*(1-가정!$C$7)</f>
         <v/>
       </c>
-      <c r="E5" s="12">
+      <c r="E5" s="29">
         <f>E4*(1-가정!$C$7)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>(+) 감가상각비</t>
         </is>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="29">
         <f>가정!$C$9*BS!E9</f>
         <v/>
       </c>
-      <c r="D6" s="12">
+      <c r="D6" s="29">
         <f>가정!$C$9*BS!F9</f>
         <v/>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="29">
         <f>가정!$C$9*BS!G9</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>(-) Capex</t>
         </is>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="29">
         <f>-가정!$C$8*IS!F4</f>
         <v/>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="29">
         <f>-가정!$C$8*IS!G4</f>
         <v/>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="29">
         <f>-가정!$C$8*IS!H4</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>(-) 순운전자본 증감</t>
         </is>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="29">
         <f>-((BS!F7+BS!F8-BS!F13)-(BS!E7+BS!E8-BS!E13))</f>
         <v/>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="29">
         <f>-((BS!G7+BS!G8-BS!G13)-(BS!F7+BS!F8-BS!F13))</f>
         <v/>
       </c>
-      <c r="E8" s="12">
+      <c r="E8" s="29">
         <f>-((BS!H7+BS!H8-BS!H13)-(BS!G7+BS!G8-BS!G13))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>FCFF</t>
         </is>
       </c>
-      <c r="C9" s="13">
+      <c r="C9" s="30">
         <f>C5+C6+C7+C8</f>
         <v/>
       </c>
-      <c r="D9" s="13">
+      <c r="D9" s="30">
         <f>D5+D6+D7+D8</f>
         <v/>
       </c>
-      <c r="E9" s="13">
+      <c r="E9" s="30">
         <f>E5+E6+E7+E8</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>할인연차 n</t>
         </is>
       </c>
-      <c r="C10" s="19" t="n">
+      <c r="C10" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="19" t="n">
+      <c r="D10" s="39" t="n">
         <v>2</v>
       </c>
-      <c r="E10" s="19" t="n">
+      <c r="E10" s="39" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>할인계수</t>
         </is>
       </c>
-      <c r="C11" s="20">
+      <c r="C11" s="40">
         <f>1/(1+가정!$C$15)^C10</f>
         <v/>
       </c>
-      <c r="D11" s="20">
+      <c r="D11" s="40">
         <f>1/(1+가정!$C$15)^D10</f>
         <v/>
       </c>
-      <c r="E11" s="20">
+      <c r="E11" s="40">
         <f>1/(1+가정!$C$15)^E10</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>PV(FCFF)</t>
         </is>
       </c>
-      <c r="C12" s="14">
+      <c r="C12" s="31">
         <f>C9*C11</f>
         <v/>
       </c>
-      <c r="D12" s="14">
+      <c r="D12" s="31">
         <f>D9*D11</f>
         <v/>
       </c>
-      <c r="E12" s="14">
+      <c r="E12" s="31">
         <f>E9*E11</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>PV(FCFF) 합계</t>
         </is>
       </c>
-      <c r="C14" s="12">
+      <c r="C14" s="29">
         <f>SUM(C12:E12)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>영구가치 (TV)</t>
         </is>
       </c>
-      <c r="C15" s="12">
+      <c r="C15" s="29">
         <f>E9*(1+가정!$C$16)/(가정!$C$15-가정!$C$16)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>PV(TV)</t>
         </is>
       </c>
-      <c r="C16" s="14">
+      <c r="C16" s="31">
         <f>C15*E11</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>기업가치 (EV)</t>
         </is>
       </c>
-      <c r="C17" s="13">
+      <c r="C17" s="30">
         <f>C14+C16</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>(-) 순차입금</t>
         </is>
       </c>
-      <c r="C18" s="12">
+      <c r="C18" s="29">
         <f>BS!E14-BS!E6</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>자기자본가치</t>
         </is>
       </c>
-      <c r="C19" s="13">
+      <c r="C19" s="30">
         <f>C17-C18</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>주식수 (백만주)</t>
-        </is>
-      </c>
-      <c r="C20" s="21">
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>주식수(백만주)</t>
+        </is>
+      </c>
+      <c r="C20" s="41">
         <f>가정!$C$17</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>주당 내재가치 (원)</t>
-        </is>
-      </c>
-      <c r="C21" s="22">
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>주당 내재가치(원)</t>
+        </is>
+      </c>
+      <c r="C21" s="42">
         <f>C19*100000000/(C20*1000000)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>(참고) 현재주가 (원)</t>
-        </is>
-      </c>
-      <c r="C22" s="23" t="n">
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>(참고) 현재주가(원)</t>
+        </is>
+      </c>
+      <c r="C22" s="43" t="n">
         <v>4000</v>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>상승여력</t>
         </is>
       </c>
-      <c r="C23" s="24">
-        <f>C21/C22-1</f>
+      <c r="C23" s="37">
+        <f>IFERROR(C21/C22-1,"-")</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="25" t="inlineStr">
-        <is>
-          <t>주당가치 민감도 (WACC × 영구성장률 g)</t>
+      <c r="B26" s="44" t="inlineStr">
+        <is>
+          <t>주당가치 민감도 — WACC × 영구성장률 g</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="C27" s="26" t="inlineStr">
-        <is>
-          <t>WACC \ g</t>
-        </is>
-      </c>
-      <c r="D27" s="27" t="n">
+      <c r="C27" s="45" t="inlineStr">
+        <is>
+          <t>WACC＼g</t>
+        </is>
+      </c>
+      <c r="D27" s="46" t="n">
         <v>0.01</v>
       </c>
-      <c r="E27" s="27" t="n">
+      <c r="E27" s="46" t="n">
         <v>0.015</v>
       </c>
-      <c r="F27" s="27" t="n">
+      <c r="F27" s="46" t="n">
         <v>0.02</v>
       </c>
-      <c r="G27" s="27" t="n">
+      <c r="G27" s="46" t="n">
         <v>0.025</v>
       </c>
-      <c r="H27" s="27" t="n">
+      <c r="H27" s="46" t="n">
         <v>0.03</v>
       </c>
     </row>
     <row r="28">
-      <c r="C28" s="28" t="n">
+      <c r="C28" s="47" t="n">
         <v>0.08</v>
       </c>
-      <c r="D28" s="29">
+      <c r="D28" s="48">
         <f>($C$9/(1+$C28)^1+$D$9/(1+$C28)^2+$E$9/(1+$C28)^3+($E$9*(1+D$27)/($C28-D$27))/(1+$C28)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
-      <c r="E28" s="29">
+      <c r="E28" s="48">
         <f>($C$9/(1+$C28)^1+$D$9/(1+$C28)^2+$E$9/(1+$C28)^3+($E$9*(1+E$27)/($C28-E$27))/(1+$C28)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
-      <c r="F28" s="29">
+      <c r="F28" s="48">
         <f>($C$9/(1+$C28)^1+$D$9/(1+$C28)^2+$E$9/(1+$C28)^3+($E$9*(1+F$27)/($C28-F$27))/(1+$C28)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
-      <c r="G28" s="29">
+      <c r="G28" s="48">
         <f>($C$9/(1+$C28)^1+$D$9/(1+$C28)^2+$E$9/(1+$C28)^3+($E$9*(1+G$27)/($C28-G$27))/(1+$C28)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
-      <c r="H28" s="29">
+      <c r="H28" s="48">
         <f>($C$9/(1+$C28)^1+$D$9/(1+$C28)^2+$E$9/(1+$C28)^3+($E$9*(1+H$27)/($C28-H$27))/(1+$C28)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="C29" s="28" t="n">
+      <c r="C29" s="47" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="D29" s="29">
+      <c r="D29" s="48">
         <f>($C$9/(1+$C29)^1+$D$9/(1+$C29)^2+$E$9/(1+$C29)^3+($E$9*(1+D$27)/($C29-D$27))/(1+$C29)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
-      <c r="E29" s="29">
+      <c r="E29" s="48">
         <f>($C$9/(1+$C29)^1+$D$9/(1+$C29)^2+$E$9/(1+$C29)^3+($E$9*(1+E$27)/($C29-E$27))/(1+$C29)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
-      <c r="F29" s="29">
+      <c r="F29" s="48">
         <f>($C$9/(1+$C29)^1+$D$9/(1+$C29)^2+$E$9/(1+$C29)^3+($E$9*(1+F$27)/($C29-F$27))/(1+$C29)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
-      <c r="G29" s="29">
+      <c r="G29" s="48">
         <f>($C$9/(1+$C29)^1+$D$9/(1+$C29)^2+$E$9/(1+$C29)^3+($E$9*(1+G$27)/($C29-G$27))/(1+$C29)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
-      <c r="H29" s="29">
+      <c r="H29" s="48">
         <f>($C$9/(1+$C29)^1+$D$9/(1+$C29)^2+$E$9/(1+$C29)^3+($E$9*(1+H$27)/($C29-H$27))/(1+$C29)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="C30" s="28" t="n">
+      <c r="C30" s="47" t="n">
         <v>0.09</v>
       </c>
-      <c r="D30" s="29">
+      <c r="D30" s="48">
         <f>($C$9/(1+$C30)^1+$D$9/(1+$C30)^2+$E$9/(1+$C30)^3+($E$9*(1+D$27)/($C30-D$27))/(1+$C30)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
-      <c r="E30" s="29">
+      <c r="E30" s="48">
         <f>($C$9/(1+$C30)^1+$D$9/(1+$C30)^2+$E$9/(1+$C30)^3+($E$9*(1+E$27)/($C30-E$27))/(1+$C30)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
-      <c r="F30" s="29">
+      <c r="F30" s="48">
         <f>($C$9/(1+$C30)^1+$D$9/(1+$C30)^2+$E$9/(1+$C30)^3+($E$9*(1+F$27)/($C30-F$27))/(1+$C30)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
-      <c r="G30" s="29">
+      <c r="G30" s="48">
         <f>($C$9/(1+$C30)^1+$D$9/(1+$C30)^2+$E$9/(1+$C30)^3+($E$9*(1+G$27)/($C30-G$27))/(1+$C30)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
-      <c r="H30" s="29">
+      <c r="H30" s="48">
         <f>($C$9/(1+$C30)^1+$D$9/(1+$C30)^2+$E$9/(1+$C30)^3+($E$9*(1+H$27)/($C30-H$27))/(1+$C30)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="C31" s="28" t="n">
+      <c r="C31" s="47" t="n">
         <v>0.095</v>
       </c>
-      <c r="D31" s="29">
+      <c r="D31" s="48">
         <f>($C$9/(1+$C31)^1+$D$9/(1+$C31)^2+$E$9/(1+$C31)^3+($E$9*(1+D$27)/($C31-D$27))/(1+$C31)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
-      <c r="E31" s="29">
+      <c r="E31" s="48">
         <f>($C$9/(1+$C31)^1+$D$9/(1+$C31)^2+$E$9/(1+$C31)^3+($E$9*(1+E$27)/($C31-E$27))/(1+$C31)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
-      <c r="F31" s="29">
+      <c r="F31" s="48">
         <f>($C$9/(1+$C31)^1+$D$9/(1+$C31)^2+$E$9/(1+$C31)^3+($E$9*(1+F$27)/($C31-F$27))/(1+$C31)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
-      <c r="G31" s="29">
+      <c r="G31" s="48">
         <f>($C$9/(1+$C31)^1+$D$9/(1+$C31)^2+$E$9/(1+$C31)^3+($E$9*(1+G$27)/($C31-G$27))/(1+$C31)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
-      <c r="H31" s="29">
+      <c r="H31" s="48">
         <f>($C$9/(1+$C31)^1+$D$9/(1+$C31)^2+$E$9/(1+$C31)^3+($E$9*(1+H$27)/($C31-H$27))/(1+$C31)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="C32" s="28" t="n">
+      <c r="C32" s="47" t="n">
         <v>0.1</v>
       </c>
-      <c r="D32" s="29">
+      <c r="D32" s="48">
         <f>($C$9/(1+$C32)^1+$D$9/(1+$C32)^2+$E$9/(1+$C32)^3+($E$9*(1+D$27)/($C32-D$27))/(1+$C32)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
-      <c r="E32" s="29">
+      <c r="E32" s="48">
         <f>($C$9/(1+$C32)^1+$D$9/(1+$C32)^2+$E$9/(1+$C32)^3+($E$9*(1+E$27)/($C32-E$27))/(1+$C32)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
-      <c r="F32" s="29">
+      <c r="F32" s="48">
         <f>($C$9/(1+$C32)^1+$D$9/(1+$C32)^2+$E$9/(1+$C32)^3+($E$9*(1+F$27)/($C32-F$27))/(1+$C32)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
-      <c r="G32" s="29">
+      <c r="G32" s="48">
         <f>($C$9/(1+$C32)^1+$D$9/(1+$C32)^2+$E$9/(1+$C32)^3+($E$9*(1+G$27)/($C32-G$27))/(1+$C32)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
       </c>
-      <c r="H32" s="29">
+      <c r="H32" s="48">
         <f>($C$9/(1+$C32)^1+$D$9/(1+$C32)^2+$E$9/(1+$C32)^3+($E$9*(1+H$27)/($C32-H$27))/(1+$C32)^3-$C$18)*100000000/($C$20*1000000)</f>
         <v/>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="D28:H32">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00F59E0B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="49" t="inlineStr">
+        <is>
+          <t>투자 요약 (Investment Summary)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>활성 시나리오 기준 · 가정 시트에서 시나리오 전환</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>시나리오</t>
+        </is>
+      </c>
+      <c r="C4" s="9">
+        <f>CHOOSE(가정!$E$1,"Base","Bull","Bear")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>기업가치 (EV, 억)</t>
+        </is>
+      </c>
+      <c r="C5" s="29">
+        <f>DCF!C17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>자기자본가치 (억)</t>
+        </is>
+      </c>
+      <c r="C6" s="29">
+        <f>DCF!C19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>목표주가</t>
+        </is>
+      </c>
+      <c r="C7" s="42">
+        <f>DCF!C21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>현재주가</t>
+        </is>
+      </c>
+      <c r="C8" s="11">
+        <f>DCF!C22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>상승여력</t>
+        </is>
+      </c>
+      <c r="C9" s="37">
+        <f>DCF!C23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>투자의견</t>
+        </is>
+      </c>
+      <c r="C10" s="15">
+        <f>IFERROR(IF(C9&gt;0.15,"매수 (Buy)",IF(C9&lt;-0.1,"매도 (Sell)","중립 (Hold)")),"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="44" t="inlineStr">
+        <is>
+          <t>매출·영업이익 추이 (억)</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>